<commit_message>
add pre week 2 files
</commit_message>
<xml_diff>
--- a/pre-week-2/homework1.xlsx
+++ b/pre-week-2/homework1.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jopso\Documents\DataAnalytics\pre-week-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23E2B55D-DE9E-4BAE-B1D0-A83CD619903F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14C3077A-5895-437E-8C34-1A7F4924E7EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{B4B97237-CFC9-442E-ACD0-29CC5E427359}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{B4B97237-CFC9-442E-ACD0-29CC5E427359}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Store_Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -130,6 +131,81 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{848BC914-120E-F404-F084-D1315C6CAACF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="38100" y="76200"/>
+          <a:ext cx="4124325" cy="2047875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>The overall average performance of the store seems to be falling around 49 monthly sales. While the store’s performance is tightly group with only one far out outliner. One value Does significantly influence the result; the 72 value in Store H greatly impacts our results. For example, our standard deviation is about 7.6 but if we take out that 72 value it drops all the way down to 2.9. Some additional information I want to add is range is also drastically impacted by outliners. Showing that all values have an impact on our data. </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -583,4 +659,14 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9631D3A-1B95-4096-92FF-B51EFBF6E833}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>